<commit_message>
product upgrades round 1/3: budget trio — charts on dashboards, clipped hero labels fixed, $0 renders as $0, dropdowns replace type-exactly fields, savings projected dates make the claim true, second-paycheck guidance, 10-debt snowball; all re-verified
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YXXCjK6mADrUUCHM2odCz1
</commit_message>
<xml_diff>
--- a/venture/07-automation/tracker/publish-queue/paycheck-budget-v1/Paycheck-Budget-System.xlsx
+++ b/venture/07-automation/tracker/publish-queue/paycheck-budget-v1/Paycheck-Budget-System.xlsx
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00;($#,##0.00)"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -132,18 +133,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -218,6 +219,200 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Your year at a glance</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Year Dashboard'!C6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3A5F"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Year Dashboard'!$B$7:$B$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Year Dashboard'!$C$7:$C$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Year Dashboard'!D6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="F2C14E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Year Dashboard'!$B$7:$B$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Year Dashboard'!$D$7:$D$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Year Dashboard'!F6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="2E7D6B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E7D6B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Year Dashboard'!$F$7:$F$18</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -507,9 +702,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E23"/>
+  <dimension ref="B2:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -580,14 +775,14 @@
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>• Debt Snowball — list debts smallest to largest; see the payoff month for each one.</t>
+          <t>• Debt Snowball — list up to 10 debts smallest to largest; see the payoff month for each one.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>• Year Dashboard — log each month once; watch your savings rate trend up.</t>
+          <t>• Year Dashboard — log each month once; watch the chart fill in and your savings rate trend up.</t>
         </is>
       </c>
     </row>
@@ -597,60 +792,107 @@
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>COLOR LEGEND</t>
+          <t>TWO OR MORE CHECKS A MONTH? (most people!)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Yellow cells = yours to edit.  Everything else calculates automatically — please don't type over it.</t>
+          <t>One tab = one paycheck. When the next check lands, make a copy of the 'Paycheck Budget' tab:</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>The numbers already in the sheet are a realistic example. Replace them with your own.</t>
+          <t>• Google Sheets: right-click the tab → Duplicate.   • Excel: right-click the tab → Move or Copy → tick 'Create a copy'.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>GOOGLE SHEETS USERS</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Rename each copy for its check (e.g. 'Aug 1 check', 'Aug 15 check') and budget that check to $0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>At the end of the month, add your checks together and log one line on the Year Dashboard.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Upload this file to Google Drive, then open it — it converts automatically and all formulas work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>COLOR LEGEND</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
+          <t>Yellow cells = yours to edit.  Everything else calculates automatically — please don't type over it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>The numbers already in the sheet are a realistic example. Replace them with your own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>GOOGLE SHEETS USERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Upload this file to Google Drive, then open it — it converts automatically and all formulas work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>The Year Dashboard chart converts to a Sheets chart too — colors may shift slightly; the numbers are identical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
           <t>Questions or a formula acting up? Message us on Etsy any time — we answer fast and we'll fix it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="B26:E26"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -658,7 +900,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -699,6 +941,13 @@
         <v>2400</v>
       </c>
     </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>One tab = one paycheck. Next check? Duplicate this tab — the how-to is on START HERE.</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -707,29 +956,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Rent / mortgage share</t>
         </is>
@@ -740,13 +989,13 @@
       <c r="D9" s="7" t="n">
         <v>950</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="11">
         <f>C9-D9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Electric</t>
         </is>
@@ -757,13 +1006,13 @@
       <c r="D10" s="7" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="11">
         <f>C10-D10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Car payment</t>
         </is>
@@ -774,13 +1023,13 @@
       <c r="D11" s="7" t="n">
         <v>310</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="11">
         <f>C11-D11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Car insurance</t>
         </is>
@@ -791,13 +1040,13 @@
       <c r="D12" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="11">
         <f>C12-D12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
@@ -808,13 +1057,13 @@
       <c r="D13" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="11">
         <f>C13-D13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Internet</t>
         </is>
@@ -825,26 +1074,26 @@
       <c r="D14" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="11">
         <f>C14-D14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="12">
         <f>SUM(C9:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="12">
         <f>SUM(D9:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="12">
         <f>C15-D15</f>
         <v/>
       </c>
@@ -857,29 +1106,29 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Groceries</t>
         </is>
@@ -890,13 +1139,13 @@
       <c r="D19" s="7" t="n">
         <v>268.51</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="11">
         <f>C19-D19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Gas</t>
         </is>
@@ -907,13 +1156,13 @@
       <c r="D20" s="7" t="n">
         <v>104.22</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="11">
         <f>C20-D20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Eating out</t>
         </is>
@@ -924,13 +1173,13 @@
       <c r="D21" s="7" t="n">
         <v>96.75</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="11">
         <f>C21-D21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Fun money</t>
         </is>
@@ -941,13 +1190,13 @@
       <c r="D22" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="11">
         <f>C22-D22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Household / misc</t>
         </is>
@@ -958,26 +1207,26 @@
       <c r="D23" s="7" t="n">
         <v>31.19</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="11">
         <f>C23-D23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="12">
         <f>SUM(C19:C23)</f>
         <v/>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="12">
         <f>SUM(D19:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="12">
         <f>C24-D24</f>
         <v/>
       </c>
@@ -990,29 +1239,29 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Emergency fund</t>
         </is>
@@ -1023,13 +1272,13 @@
       <c r="D28" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="E28" s="10">
+      <c r="E28" s="11">
         <f>C28-D28</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Extra to smallest debt</t>
         </is>
@@ -1040,32 +1289,32 @@
       <c r="D29" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="E29" s="10">
+      <c r="E29" s="11">
         <f>C29-D29</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="12">
         <f>SUM(C28:C29)</f>
         <v/>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="12">
         <f>SUM(D28:D29)</f>
         <v/>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="12">
         <f>C30-D30</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>THE BOTTOM LINE</t>
         </is>
@@ -1077,7 +1326,7 @@
           <t>Left to Assign (planned) — get this to $0</t>
         </is>
       </c>
-      <c r="C33" s="13">
+      <c r="E33" s="14">
         <f>C5-C15-C24-C30</f>
         <v/>
       </c>
@@ -1088,27 +1337,30 @@
           <t>Actually remaining (real money right now)</t>
         </is>
       </c>
-      <c r="C34" s="13">
+      <c r="E34" s="14">
         <f>C5-D15-D24-D30</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Tip: 'Left to Assign' at $0 means every dollar has a job before you spend it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="B33:D33"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B34:D34"/>
     <mergeCell ref="B32:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1116,9 +1368,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:G14"/>
+  <dimension ref="B2:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1138,7 +1390,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>List debts SMALLEST balance first. Put your monthly extra payment in the yellow cell — it attacks the top debt.</t>
         </is>
@@ -1155,39 +1407,39 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Debt</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Min payment</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>You pay</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Months to payoff</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Store card</t>
         </is>
@@ -1201,17 +1453,17 @@
       <c r="E8" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="F8" s="10">
-        <f>E8+IF(ROW()=8,$C$5,0)</f>
+      <c r="F8" s="11">
+        <f>IF(OR($C8="",$C8=0),"",E8+IF(ROW()=8,$C$5,0))</f>
         <v/>
       </c>
       <c r="G8" s="16">
-        <f>IFERROR(ROUNDUP(NPER(D8/12,-F8,C8),0),"raise payment")</f>
+        <f>IF(OR($C8="",$C8=0),"",IFERROR(ROUNDUP(NPER(D8/12,-F8,C8),0),"raise payment"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Credit card</t>
         </is>
@@ -1225,17 +1477,17 @@
       <c r="E9" s="7" t="n">
         <v>75</v>
       </c>
-      <c r="F9" s="10">
-        <f>E9+IF(ROW()=8,$C$5,0)</f>
+      <c r="F9" s="11">
+        <f>IF(OR($C9="",$C9=0),"",E9+IF(ROW()=8,$C$5,0))</f>
         <v/>
       </c>
       <c r="G9" s="16">
-        <f>IFERROR(ROUNDUP(NPER(D9/12,-F9,C9),0),"raise payment")</f>
+        <f>IF(OR($C9="",$C9=0),"",IFERROR(ROUNDUP(NPER(D9/12,-F9,C9),0),"raise payment"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Car loan</t>
         </is>
@@ -1249,42 +1501,140 @@
       <c r="E10" s="7" t="n">
         <v>310</v>
       </c>
-      <c r="F10" s="10">
-        <f>E10+IF(ROW()=8,$C$5,0)</f>
+      <c r="F10" s="11">
+        <f>IF(OR($C10="",$C10=0),"",E10+IF(ROW()=8,$C$5,0))</f>
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>IFERROR(ROUNDUP(NPER(D10/12,-F10,C10),0),"raise payment")</f>
+        <f>IF(OR($C10="",$C10=0),"",IFERROR(ROUNDUP(NPER(D10/12,-F10,C10),0),"raise payment"))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="11">
+        <f>IF(OR($C11="",$C11=0),"",E11+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G11" s="16">
+        <f>IF(OR($C11="",$C11=0),"",IFERROR(ROUNDUP(NPER(D11/12,-F11,C11),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="11">
+        <f>IF(OR($C12="",$C12=0),"",E12+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G12" s="16">
+        <f>IF(OR($C12="",$C12=0),"",IFERROR(ROUNDUP(NPER(D12/12,-F12,C12),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="11">
+        <f>IF(OR($C13="",$C13=0),"",E13+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G13" s="16">
+        <f>IF(OR($C13="",$C13=0),"",IFERROR(ROUNDUP(NPER(D13/12,-F13,C13),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="11">
+        <f>IF(OR($C14="",$C14=0),"",E14+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G14" s="16">
+        <f>IF(OR($C14="",$C14=0),"",IFERROR(ROUNDUP(NPER(D14/12,-F14,C14),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="11">
+        <f>IF(OR($C15="",$C15=0),"",E15+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G15" s="16">
+        <f>IF(OR($C15="",$C15=0),"",IFERROR(ROUNDUP(NPER(D15/12,-F15,C15),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="11">
+        <f>IF(OR($C16="",$C16=0),"",E16+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G16" s="16">
+        <f>IF(OR($C16="",$C16=0),"",IFERROR(ROUNDUP(NPER(D16/12,-F16,C16),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="11">
+        <f>IF(OR($C17="",$C17=0),"",E17+IF(ROW()=8,$C$5,0))</f>
+        <v/>
+      </c>
+      <c r="G17" s="16">
+        <f>IF(OR($C17="",$C17=0),"",IFERROR(ROUNDUP(NPER(D17/12,-F17,C17),0),"raise payment"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C11" s="11">
-        <f>SUM(C8:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="11">
-        <f>SUM(F8:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="17" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="14" t="inlineStr">
+      <c r="C18" s="12">
+        <f>SUM(C8:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="12">
+        <f>SUM(F8:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="17" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>When a debt hits $0, roll its whole 'You pay' amount onto the next debt down. That's the snowball.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="14" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>"raise payment" means the payment doesn't cover the interest — increase it.</t>
         </is>
@@ -1295,6 +1645,7 @@
     <mergeCell ref="B2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1302,7 +1653,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1323,41 +1674,41 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Once a month, copy your totals here (2 minutes). Watch the savings-rate column — that's the number that changes your life.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Spent</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Saved</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Savings rate</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
@@ -1371,7 +1722,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
@@ -1385,7 +1736,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
@@ -1399,7 +1750,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
@@ -1413,7 +1764,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>May</t>
         </is>
@@ -1427,7 +1778,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
@@ -1441,7 +1792,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
@@ -1455,7 +1806,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
@@ -1475,7 +1826,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
@@ -1489,7 +1840,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
@@ -1503,7 +1854,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
@@ -1517,7 +1868,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
@@ -1531,20 +1882,20 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Year total</t>
         </is>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="12">
         <f>SUM(C7:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="12">
         <f>SUM(D7:D18)</f>
         <v/>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="12">
         <f>SUM(E7:E18)</f>
         <v/>
       </c>
@@ -1554,7 +1905,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>August row is a worked example — clear it and enter your own months.</t>
         </is>
@@ -1565,5 +1916,7 @@
     <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>